<commit_message>
Most recent ESCAPE results
</commit_message>
<xml_diff>
--- a/hexaly_benchmarking_results/known_n.xlsx
+++ b/hexaly_benchmarking_results/known_n.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="10">
   <si>
     <t>Accuracy</t>
   </si>
@@ -456,10 +456,10 @@
         <v>-86</v>
       </c>
       <c r="C3">
-        <v>-86.00000000000003</v>
+        <v>-86.00000000000006</v>
       </c>
       <c r="D3">
-        <v>3.304849933767907E-14</v>
+        <v>6.609699867535812E-14</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -473,13 +473,13 @@
         <v>40</v>
       </c>
       <c r="B4">
-        <v>-145</v>
+        <v>-145.0000000000001</v>
       </c>
       <c r="C4">
         <v>-145.0000000000001</v>
       </c>
       <c r="D4">
-        <v>3.920235783503999E-14</v>
+        <v>0</v>
       </c>
       <c r="E4">
         <v>0</v>
@@ -533,13 +533,13 @@
         <v>20</v>
       </c>
       <c r="B7">
-        <v>-868.0000000000001</v>
+        <v>-868</v>
       </c>
       <c r="C7">
-        <v>-868.0000000000001</v>
+        <v>-868.0202623340165</v>
       </c>
       <c r="D7">
-        <v>0</v>
+        <v>0.002334315786822284</v>
       </c>
       <c r="E7">
         <v>0</v>
@@ -553,13 +553,13 @@
         <v>17</v>
       </c>
       <c r="B8">
-        <v>-1060.5</v>
+        <v>-1060.500000000016</v>
       </c>
       <c r="C8">
-        <v>-1060.500001869311</v>
+        <v>-1060.500000000355</v>
       </c>
       <c r="D8">
-        <v>1.76266976648055E-07</v>
+        <v>3.194594779917985E-11</v>
       </c>
       <c r="E8">
         <v>0</v>
@@ -573,10 +573,10 @@
         <v>15</v>
       </c>
       <c r="B9">
-        <v>-1254.000000000003</v>
+        <v>-1254.000000000001</v>
       </c>
       <c r="C9">
-        <v>-1254.000000000003</v>
+        <v>-1254.000000000001</v>
       </c>
       <c r="D9">
         <v>0</v>
@@ -613,13 +613,13 @@
         <v>12</v>
       </c>
       <c r="B11">
-        <v>-1635.000000000007</v>
+        <v>-1634.999999999998</v>
       </c>
       <c r="C11">
-        <v>-1635.000002568875</v>
+        <v>-1635.000000000048</v>
       </c>
       <c r="D11">
-        <v>1.571172676681431E-07</v>
+        <v>3.101182239990168E-12</v>
       </c>
       <c r="E11">
         <v>0</v>
@@ -653,10 +653,10 @@
         <v>9</v>
       </c>
       <c r="B13">
-        <v>-2218.000000000187</v>
+        <v>-2218.000000000007</v>
       </c>
       <c r="C13">
-        <v>-2218.000000000187</v>
+        <v>-2218.000000000007</v>
       </c>
       <c r="D13">
         <v>0</v>
@@ -682,7 +682,7 @@
         <v>0</v>
       </c>
       <c r="E14">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F14" t="s">
         <v>6</v>
@@ -693,13 +693,13 @@
         <v>7</v>
       </c>
       <c r="B15">
-        <v>-2937.500136454142</v>
+        <v>-2937.500157055813</v>
       </c>
       <c r="C15">
         <v>-11664.00000000002</v>
       </c>
       <c r="D15">
-        <v>74.81567098376082</v>
+        <v>74.81567080713471</v>
       </c>
       <c r="E15">
         <v>300</v>
@@ -713,13 +713,13 @@
         <v>6</v>
       </c>
       <c r="B16">
-        <v>-3499.000134959687</v>
+        <v>-3499.000255781522</v>
       </c>
       <c r="C16">
         <v>-14187.00000000003</v>
       </c>
       <c r="D16">
-        <v>75.33657478706081</v>
+        <v>75.33657393542316</v>
       </c>
       <c r="E16">
         <v>300</v>
@@ -733,13 +733,13 @@
         <v>5</v>
       </c>
       <c r="B17">
-        <v>-4210.000100763938</v>
+        <v>-4211.000243740127</v>
       </c>
       <c r="C17">
-        <v>-17566.00000000004</v>
+        <v>-17531.00000000004</v>
       </c>
       <c r="D17">
-        <v>76.03324546986265</v>
+        <v>75.97969172471555</v>
       </c>
       <c r="E17">
         <v>300</v>
@@ -753,13 +753,13 @@
         <v>4</v>
       </c>
       <c r="B18">
-        <v>-4942.000334297435</v>
+        <v>-4763.000289078626</v>
       </c>
       <c r="C18">
-        <v>-19514.00000000002</v>
+        <v>-19539.00000000002</v>
       </c>
       <c r="D18">
-        <v>74.67459088706863</v>
+        <v>75.62311126936578</v>
       </c>
       <c r="E18">
         <v>300</v>
@@ -773,13 +773,13 @@
         <v>3</v>
       </c>
       <c r="B19">
-        <v>-6164.000399892392</v>
+        <v>-6371.000435102151</v>
       </c>
       <c r="C19">
-        <v>-20724.00000000004</v>
+        <v>-20739.00000000004</v>
       </c>
       <c r="D19">
-        <v>70.25670526977234</v>
+        <v>69.28009819614186</v>
       </c>
       <c r="E19">
         <v>300</v>
@@ -793,13 +793,13 @@
         <v>2</v>
       </c>
       <c r="B20">
-        <v>-7701.000434593269</v>
+        <v>-7818.000162787889</v>
       </c>
       <c r="C20">
-        <v>-23593.00000000009</v>
+        <v>-23598.00000000009</v>
       </c>
       <c r="D20">
-        <v>67.35896056205976</v>
+        <v>66.87007304522477</v>
       </c>
       <c r="E20">
         <v>300</v>
@@ -813,13 +813,13 @@
         <v>1</v>
       </c>
       <c r="B21">
-        <v>-11738.22459070672</v>
+        <v>-11068.10121677245</v>
       </c>
       <c r="C21">
         <v>-25755</v>
       </c>
       <c r="D21">
-        <v>54.42351158723851</v>
+        <v>57.02542723054766</v>
       </c>
       <c r="E21">
         <v>300</v>
@@ -903,10 +903,10 @@
         <v>40</v>
       </c>
       <c r="B4">
-        <v>-145</v>
+        <v>-145.0000035456657</v>
       </c>
       <c r="C4">
-        <v>-145</v>
+        <v>-145.0000035456657</v>
       </c>
       <c r="D4">
         <v>0</v>
@@ -923,13 +923,13 @@
         <v>30</v>
       </c>
       <c r="B5">
-        <v>-450.9999999999991</v>
+        <v>-451</v>
       </c>
       <c r="C5">
-        <v>-451.0000000000003</v>
+        <v>-451.0000000000001</v>
       </c>
       <c r="D5">
-        <v>2.646811077775981E-13</v>
+        <v>1.260386227512373E-14</v>
       </c>
       <c r="E5">
         <v>0</v>
@@ -943,13 +943,13 @@
         <v>24</v>
       </c>
       <c r="B6">
-        <v>-659.0000000003594</v>
+        <v>-658.9999999999989</v>
       </c>
       <c r="C6">
-        <v>-659.0000000003594</v>
+        <v>-659.0000000004791</v>
       </c>
       <c r="D6">
-        <v>0</v>
+        <v>7.28699852102818E-11</v>
       </c>
       <c r="E6">
         <v>0</v>
@@ -963,16 +963,16 @@
         <v>20</v>
       </c>
       <c r="B7">
-        <v>-868.0000035601394</v>
+        <v>-868.0000000043406</v>
       </c>
       <c r="C7">
-        <v>-868.0000065783852</v>
+        <v>-868.0000083491861</v>
       </c>
       <c r="D7">
-        <v>3.47724170220128E-07</v>
+        <v>9.613877306767098E-07</v>
       </c>
       <c r="E7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F7" t="s">
         <v>6</v>
@@ -983,13 +983,13 @@
         <v>17</v>
       </c>
       <c r="B8">
-        <v>-1060.500011716563</v>
+        <v>-1060.500012055399</v>
       </c>
       <c r="C8">
-        <v>-1060.500011805115</v>
+        <v>-1060.500016475598</v>
       </c>
       <c r="D8">
-        <v>8.350006014522974E-09</v>
+        <v>4.168032769097318E-07</v>
       </c>
       <c r="E8">
         <v>4</v>
@@ -1003,16 +1003,16 @@
         <v>15</v>
       </c>
       <c r="B9">
-        <v>-1254.000009846905</v>
+        <v>-1254.000006284345</v>
       </c>
       <c r="C9">
-        <v>-1254.000009846905</v>
+        <v>-1254.000010053599</v>
       </c>
       <c r="D9">
-        <v>0</v>
+        <v>3.005784772933242E-07</v>
       </c>
       <c r="E9">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F9" t="s">
         <v>6</v>
@@ -1023,16 +1023,16 @@
         <v>13</v>
       </c>
       <c r="B10">
-        <v>-1449.000011087917</v>
+        <v>-1449.000010879016</v>
       </c>
       <c r="C10">
-        <v>-1449.000011087917</v>
+        <v>-1449.000010879016</v>
       </c>
       <c r="D10">
         <v>0</v>
       </c>
       <c r="E10">
-        <v>34</v>
+        <v>64</v>
       </c>
       <c r="F10" t="s">
         <v>6</v>
@@ -1043,19 +1043,19 @@
         <v>12</v>
       </c>
       <c r="B11">
-        <v>-1635.000027460446</v>
+        <v>-1635.00002838934</v>
       </c>
       <c r="C11">
-        <v>-1642.999999999979</v>
+        <v>-1635.00002838934</v>
       </c>
       <c r="D11">
-        <v>0.4869125100141888</v>
+        <v>0</v>
       </c>
       <c r="E11">
-        <v>300</v>
+        <v>263</v>
       </c>
       <c r="F11" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -1063,13 +1063,13 @@
         <v>10</v>
       </c>
       <c r="B12">
-        <v>-2002.000007186359</v>
+        <v>-2002.000007198596</v>
       </c>
       <c r="C12">
-        <v>-2469.999999999952</v>
+        <v>-2469.999999999876</v>
       </c>
       <c r="D12">
-        <v>18.94736813010534</v>
+        <v>18.94736812960744</v>
       </c>
       <c r="E12">
         <v>300</v>
@@ -1083,13 +1083,13 @@
         <v>9</v>
       </c>
       <c r="B13">
-        <v>-2182.000011005578</v>
+        <v>-2214.792097351755</v>
       </c>
       <c r="C13">
-        <v>-2517.999999999949</v>
+        <v>-2517.999999999934</v>
       </c>
       <c r="D13">
-        <v>13.34392331192919</v>
+        <v>12.04161646736246</v>
       </c>
       <c r="E13">
         <v>300</v>
@@ -1103,13 +1103,13 @@
         <v>8</v>
       </c>
       <c r="B14">
-        <v>-2587.000007149653</v>
+        <v>-2587.000007165996</v>
       </c>
       <c r="C14">
-        <v>-3234.999999999523</v>
+        <v>-3234.999999998702</v>
       </c>
       <c r="D14">
-        <v>20.03091168006076</v>
+        <v>20.03091167953527</v>
       </c>
       <c r="E14">
         <v>300</v>
@@ -1123,13 +1123,13 @@
         <v>7</v>
       </c>
       <c r="B15">
-        <v>-2935.423997013816</v>
+        <v>-2934.262868179775</v>
       </c>
       <c r="C15">
-        <v>-3371.99999999998</v>
+        <v>-3371.999999999989</v>
       </c>
       <c r="D15">
-        <v>12.94709380148774</v>
+        <v>12.98152822717129</v>
       </c>
       <c r="E15">
         <v>300</v>
@@ -1143,13 +1143,13 @@
         <v>6</v>
       </c>
       <c r="B16">
-        <v>-3499.000011186125</v>
+        <v>-3499.000010613431</v>
       </c>
       <c r="C16">
-        <v>-11130.17347597485</v>
+        <v>-7593.576308782231</v>
       </c>
       <c r="D16">
-        <v>68.56293373379198</v>
+        <v>53.92157965718053</v>
       </c>
       <c r="E16">
         <v>300</v>
@@ -1163,13 +1163,13 @@
         <v>5</v>
       </c>
       <c r="B17">
-        <v>-4210</v>
+        <v>-4211.000007167921</v>
       </c>
       <c r="C17">
-        <v>-27110</v>
+        <v>-27075</v>
       </c>
       <c r="D17">
-        <v>84.47067502766507</v>
+        <v>84.44690671406123</v>
       </c>
       <c r="E17">
         <v>300</v>
@@ -1183,13 +1183,13 @@
         <v>4</v>
       </c>
       <c r="B18">
-        <v>-4941.997911415068</v>
+        <v>-4763.000007070595</v>
       </c>
       <c r="C18">
-        <v>-26990</v>
+        <v>-27015</v>
       </c>
       <c r="D18">
-        <v>81.68952237341583</v>
+        <v>82.36905420295912</v>
       </c>
       <c r="E18">
         <v>300</v>
@@ -1203,13 +1203,13 @@
         <v>3</v>
       </c>
       <c r="B19">
-        <v>-6164.00000687087</v>
+        <v>-6344.000002643128</v>
       </c>
       <c r="C19">
-        <v>-26640</v>
+        <v>-26655</v>
       </c>
       <c r="D19">
-        <v>76.86186183607032</v>
+        <v>76.19958730953618</v>
       </c>
       <c r="E19">
         <v>300</v>
@@ -1223,19 +1223,19 @@
         <v>2</v>
       </c>
       <c r="B20">
-        <v>343.0000000000982</v>
+        <v>-7567.83261715334</v>
       </c>
       <c r="C20">
-        <v>-26485</v>
-      </c>
-      <c r="D20" t="s">
-        <v>8</v>
+        <v>-26490</v>
+      </c>
+      <c r="D20">
+        <v>71.43136044864727</v>
       </c>
       <c r="E20">
         <v>300</v>
       </c>
       <c r="F20" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="21" spans="1:6">
@@ -1243,7 +1243,7 @@
         <v>1</v>
       </c>
       <c r="B21">
-        <v>-5876.379236389156</v>
+        <v>877</v>
       </c>
       <c r="C21">
         <v>-25755</v>
@@ -1333,13 +1333,13 @@
         <v>40</v>
       </c>
       <c r="B4">
-        <v>-145</v>
+        <v>-145.0000000000001</v>
       </c>
       <c r="C4">
-        <v>-145</v>
+        <v>-145.0000000000001</v>
       </c>
       <c r="D4">
-        <v>1.960117891752E-14</v>
+        <v>0</v>
       </c>
       <c r="E4">
         <v>0</v>
@@ -1353,13 +1353,13 @@
         <v>30</v>
       </c>
       <c r="B5">
+        <v>-451.0000000000002</v>
+      </c>
+      <c r="C5">
         <v>-451.0000000000003</v>
       </c>
-      <c r="C5">
-        <v>-451.0000000000005</v>
-      </c>
       <c r="D5">
-        <v>2.520772455024743E-14</v>
+        <v>1.260386227512372E-14</v>
       </c>
       <c r="E5">
         <v>0</v>
@@ -1373,13 +1373,13 @@
         <v>24</v>
       </c>
       <c r="B6">
-        <v>-659.0000000000978</v>
+        <v>-659.0000000000005</v>
       </c>
       <c r="C6">
-        <v>-659.0000000002278</v>
+        <v>-659.0000000000006</v>
       </c>
       <c r="D6">
-        <v>1.973562099445884E-11</v>
+        <v>1.725141695320424E-14</v>
       </c>
       <c r="E6">
         <v>0</v>
@@ -1393,16 +1393,16 @@
         <v>20</v>
       </c>
       <c r="B7">
-        <v>-868.0000107691252</v>
+        <v>-868.0000160197219</v>
       </c>
       <c r="C7">
-        <v>-868.0000107691252</v>
+        <v>-868.0000160197219</v>
       </c>
       <c r="D7">
         <v>0</v>
       </c>
       <c r="E7">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="F7" t="s">
         <v>6</v>
@@ -1413,19 +1413,19 @@
         <v>17</v>
       </c>
       <c r="B8">
-        <v>-1060.500020243962</v>
+        <v>-1060.500018879588</v>
       </c>
       <c r="C8">
-        <v>-1108.580952380951</v>
+        <v>-1060.500018879588</v>
       </c>
       <c r="D8">
-        <v>4.337160225757389</v>
+        <v>0</v>
       </c>
       <c r="E8">
-        <v>300</v>
+        <v>175</v>
       </c>
       <c r="F8" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -1433,19 +1433,19 @@
         <v>15</v>
       </c>
       <c r="B9">
-        <v>-1254.000011113745</v>
+        <v>-1254.000011184923</v>
       </c>
       <c r="C9">
-        <v>-1254.000011113745</v>
+        <v>-1262</v>
       </c>
       <c r="D9">
-        <v>0</v>
+        <v>0.6339135352676194</v>
       </c>
       <c r="E9">
-        <v>113</v>
+        <v>300</v>
       </c>
       <c r="F9" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -1453,13 +1453,13 @@
         <v>13</v>
       </c>
       <c r="B10">
-        <v>-1449.000011097066</v>
+        <v>-1449.000011171598</v>
       </c>
       <c r="C10">
-        <v>-1453.000000000041</v>
+        <v>-1704.999999999796</v>
       </c>
       <c r="D10">
-        <v>0.2752917345474659</v>
+        <v>15.01466210136237</v>
       </c>
       <c r="E10">
         <v>300</v>
@@ -1473,13 +1473,13 @@
         <v>12</v>
       </c>
       <c r="B11">
-        <v>-1635.000028178484</v>
+        <v>-1635.000028908659</v>
       </c>
       <c r="C11">
-        <v>-1832.227016950236</v>
+        <v>-1700</v>
       </c>
       <c r="D11">
-        <v>10.76433143639805</v>
+        <v>3.823527711255377</v>
       </c>
       <c r="E11">
         <v>300</v>
@@ -1493,13 +1493,13 @@
         <v>10</v>
       </c>
       <c r="B12">
-        <v>-2002.000007096792</v>
+        <v>-2001.999848598414</v>
       </c>
       <c r="C12">
-        <v>-2885.224314927595</v>
+        <v>-2937.802959907597</v>
       </c>
       <c r="D12">
-        <v>30.61198060965903</v>
+        <v>31.85384193835167</v>
       </c>
       <c r="E12">
         <v>300</v>
@@ -1513,13 +1513,13 @@
         <v>9</v>
       </c>
       <c r="B13">
-        <v>-2218.000008917436</v>
+        <v>-2218.000011088411</v>
       </c>
       <c r="C13">
-        <v>-3954.233891787894</v>
+        <v>-4036.718166019533</v>
       </c>
       <c r="D13">
-        <v>43.90822420687475</v>
+        <v>45.05437536464172</v>
       </c>
       <c r="E13">
         <v>300</v>
@@ -1533,13 +1533,13 @@
         <v>8</v>
       </c>
       <c r="B14">
-        <v>-2587.000007179574</v>
+        <v>-2587.000007184351</v>
       </c>
       <c r="C14">
-        <v>-7906.355157097832</v>
+        <v>-7763.619539464617</v>
       </c>
       <c r="D14">
-        <v>67.27948649186185</v>
+        <v>66.67791364538257</v>
       </c>
       <c r="E14">
         <v>300</v>
@@ -1553,13 +1553,13 @@
         <v>7</v>
       </c>
       <c r="B15">
-        <v>-2936.566193933411</v>
+        <v>-2933.406112432342</v>
       </c>
       <c r="C15">
-        <v>-9708.015219157256</v>
+        <v>-10041.83681899469</v>
       </c>
       <c r="D15">
-        <v>69.75111670469413</v>
+        <v>70.78815195559001</v>
       </c>
       <c r="E15">
         <v>300</v>
@@ -1573,13 +1573,13 @@
         <v>6</v>
       </c>
       <c r="B16">
-        <v>-3499.000010174158</v>
+        <v>-3499.000011151707</v>
       </c>
       <c r="C16">
-        <v>-14707.61866693906</v>
+        <v>-17097.52069760642</v>
       </c>
       <c r="D16">
-        <v>76.20960884687959</v>
+        <v>79.53504444862844</v>
       </c>
       <c r="E16">
         <v>300</v>
@@ -1593,13 +1593,13 @@
         <v>5</v>
       </c>
       <c r="B17">
-        <v>-4210</v>
+        <v>-4211.000007079504</v>
       </c>
       <c r="C17">
-        <v>-22546.628143935</v>
+        <v>-23291.02659388755</v>
       </c>
       <c r="D17">
-        <v>81.3275848915241</v>
+        <v>81.92007557028582</v>
       </c>
       <c r="E17">
         <v>300</v>
@@ -1613,13 +1613,13 @@
         <v>4</v>
       </c>
       <c r="B18">
-        <v>-4942.000010529676</v>
+        <v>-4763.000006256601</v>
       </c>
       <c r="C18">
-        <v>-26990</v>
+        <v>-27015</v>
       </c>
       <c r="D18">
-        <v>81.68951459603677</v>
+        <v>82.36905420597222</v>
       </c>
       <c r="E18">
         <v>300</v>
@@ -1633,13 +1633,13 @@
         <v>3</v>
       </c>
       <c r="B19">
-        <v>-6164.000006015738</v>
+        <v>-6371.000010875239</v>
       </c>
       <c r="C19">
-        <v>-26640</v>
+        <v>-26655</v>
       </c>
       <c r="D19">
-        <v>76.86186183928025</v>
+        <v>76.0982929623889</v>
       </c>
       <c r="E19">
         <v>300</v>
@@ -1653,13 +1653,13 @@
         <v>2</v>
       </c>
       <c r="B20">
-        <v>-7701.000006803318</v>
+        <v>-7850.000005262159</v>
       </c>
       <c r="C20">
-        <v>-26485</v>
+        <v>-26490</v>
       </c>
       <c r="D20">
-        <v>70.9231640294381</v>
+        <v>70.36617589557508</v>
       </c>
       <c r="E20">
         <v>300</v>
@@ -1673,13 +1673,13 @@
         <v>1</v>
       </c>
       <c r="B21">
-        <v>-13018.99999861548</v>
+        <v>-13018.99984637278</v>
       </c>
       <c r="C21">
         <v>-25755</v>
       </c>
       <c r="D21">
-        <v>49.45059212341108</v>
+        <v>49.45059271453008</v>
       </c>
       <c r="E21">
         <v>300</v>
@@ -1743,13 +1743,13 @@
         <v>60</v>
       </c>
       <c r="B3">
-        <v>-86</v>
+        <v>-86.00000000000003</v>
       </c>
       <c r="C3">
-        <v>-86.00000000000001</v>
+        <v>-86.00000000000003</v>
       </c>
       <c r="D3">
-        <v>1.652424966883954E-14</v>
+        <v>0</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -1783,13 +1783,13 @@
         <v>30</v>
       </c>
       <c r="B5">
-        <v>-451</v>
+        <v>-450.9995000645418</v>
       </c>
       <c r="C5">
-        <v>-451</v>
+        <v>-451.0001483518363</v>
       </c>
       <c r="D5">
-        <v>0</v>
+        <v>0.0001437443639257585</v>
       </c>
       <c r="E5">
         <v>0</v>
@@ -1843,16 +1843,16 @@
         <v>17</v>
       </c>
       <c r="B8">
-        <v>-1060.500000000001</v>
+        <v>-1060.499999999991</v>
       </c>
       <c r="C8">
-        <v>-1060.500000000001</v>
+        <v>-1060.499999999991</v>
       </c>
       <c r="D8">
         <v>0</v>
       </c>
       <c r="E8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F8" t="s">
         <v>6</v>
@@ -1863,10 +1863,10 @@
         <v>15</v>
       </c>
       <c r="B9">
-        <v>-1254</v>
+        <v>-1253.999999999999</v>
       </c>
       <c r="C9">
-        <v>-1254</v>
+        <v>-1253.999999999999</v>
       </c>
       <c r="D9">
         <v>0</v>
@@ -1892,7 +1892,7 @@
         <v>0</v>
       </c>
       <c r="E10">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F10" t="s">
         <v>6</v>
@@ -1903,16 +1903,16 @@
         <v>12</v>
       </c>
       <c r="B11">
-        <v>-1635</v>
+        <v>-1635.000000000205</v>
       </c>
       <c r="C11">
-        <v>-1635</v>
+        <v>-1635.000000000205</v>
       </c>
       <c r="D11">
         <v>0</v>
       </c>
       <c r="E11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F11" t="s">
         <v>6</v>
@@ -1932,7 +1932,7 @@
         <v>0</v>
       </c>
       <c r="E12">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="F12" t="s">
         <v>6</v>
@@ -1972,7 +1972,7 @@
         <v>0</v>
       </c>
       <c r="E14">
-        <v>9</v>
+        <v>34</v>
       </c>
       <c r="F14" t="s">
         <v>6</v>
@@ -1983,16 +1983,16 @@
         <v>7</v>
       </c>
       <c r="B15">
-        <v>-2937.500196823912</v>
+        <v>-2937.5</v>
       </c>
       <c r="C15">
-        <v>-2937.500196823917</v>
+        <v>-2937.5</v>
       </c>
       <c r="D15">
-        <v>1.548075984397026E-13</v>
+        <v>0</v>
       </c>
       <c r="E15">
-        <v>76</v>
+        <v>94</v>
       </c>
       <c r="F15" t="s">
         <v>6</v>
@@ -2003,16 +2003,16 @@
         <v>6</v>
       </c>
       <c r="B16">
-        <v>-3499</v>
+        <v>-3499.000241669576</v>
       </c>
       <c r="C16">
-        <v>-3499</v>
+        <v>-3499.000244261619</v>
       </c>
       <c r="D16">
-        <v>0</v>
+        <v>7.407952096901042E-08</v>
       </c>
       <c r="E16">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="F16" t="s">
         <v>6</v>
@@ -2023,13 +2023,13 @@
         <v>5</v>
       </c>
       <c r="B17">
-        <v>-4165</v>
+        <v>-4119.000348170899</v>
       </c>
       <c r="C17">
-        <v>-4209.999999999</v>
+        <v>-4210.99999999377</v>
       </c>
       <c r="D17">
-        <v>1.068883610427818</v>
+        <v>2.184745946877392</v>
       </c>
       <c r="E17">
         <v>300</v>
@@ -2043,19 +2043,19 @@
         <v>4</v>
       </c>
       <c r="B18">
-        <v>-4938.000291311813</v>
+        <v>-4763.000320036102</v>
       </c>
       <c r="C18">
-        <v>-4941.999999976424</v>
+        <v>-4763.000320036102</v>
       </c>
       <c r="D18">
-        <v>0.08093299604673994</v>
+        <v>0</v>
       </c>
       <c r="E18">
-        <v>300</v>
+        <v>246</v>
       </c>
       <c r="F18" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="19" spans="1:6">
@@ -2063,19 +2063,19 @@
         <v>3</v>
       </c>
       <c r="B19">
-        <v>-6164</v>
+        <v>-6191.000473068396</v>
       </c>
       <c r="C19">
-        <v>-6164</v>
+        <v>-19213.93877550212</v>
       </c>
       <c r="D19">
-        <v>0</v>
+        <v>67.77859789497218</v>
       </c>
       <c r="E19">
-        <v>80</v>
+        <v>300</v>
       </c>
       <c r="F19" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="20" spans="1:6">
@@ -2083,19 +2083,19 @@
         <v>2</v>
       </c>
       <c r="B20">
-        <v>1515</v>
+        <v>-4114.087816757833</v>
       </c>
       <c r="C20">
-        <v>-23593.00000000009</v>
-      </c>
-      <c r="D20" t="s">
-        <v>8</v>
+        <v>-23598.00000000009</v>
+      </c>
+      <c r="D20">
+        <v>82.5659470431485</v>
       </c>
       <c r="E20">
         <v>300</v>
       </c>
       <c r="F20" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="21" spans="1:6">
@@ -2196,10 +2196,10 @@
         <v>-145.0000000000001</v>
       </c>
       <c r="C4">
-        <v>-145.0000000000001</v>
+        <v>-145.0000008254828</v>
       </c>
       <c r="D4">
-        <v>1.960117891751999E-14</v>
+        <v>5.692984601490828E-07</v>
       </c>
       <c r="E4">
         <v>0</v>
@@ -2253,13 +2253,13 @@
         <v>20</v>
       </c>
       <c r="B7">
-        <v>-868.0000000000001</v>
+        <v>-868.000000000001</v>
       </c>
       <c r="C7">
-        <v>-868.0000271320782</v>
+        <v>-868.0000105198319</v>
       </c>
       <c r="D7">
-        <v>3.125815353521475E-06</v>
+        <v>1.211962068282054E-06</v>
       </c>
       <c r="E7">
         <v>1</v>
@@ -2273,16 +2273,16 @@
         <v>17</v>
       </c>
       <c r="B8">
-        <v>-1060.500048988422</v>
+        <v>-1060.500038374746</v>
       </c>
       <c r="C8">
-        <v>-1060.500048988422</v>
+        <v>-1060.500038374746</v>
       </c>
       <c r="D8">
         <v>0</v>
       </c>
       <c r="E8">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="F8" t="s">
         <v>6</v>
@@ -2296,13 +2296,13 @@
         <v>-1254</v>
       </c>
       <c r="C9">
-        <v>-1254.000000000003</v>
+        <v>-1254</v>
       </c>
       <c r="D9">
-        <v>2.538462086288071E-13</v>
+        <v>0</v>
       </c>
       <c r="E9">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="F9" t="s">
         <v>6</v>
@@ -2313,16 +2313,16 @@
         <v>13</v>
       </c>
       <c r="B10">
-        <v>-1449.000076029421</v>
+        <v>-1449.000083030363</v>
       </c>
       <c r="C10">
-        <v>-1449.000076029421</v>
+        <v>-1449.000083030363</v>
       </c>
       <c r="D10">
         <v>0</v>
       </c>
       <c r="E10">
-        <v>96</v>
+        <v>32</v>
       </c>
       <c r="F10" t="s">
         <v>6</v>
@@ -2333,16 +2333,16 @@
         <v>12</v>
       </c>
       <c r="B11">
-        <v>-1635.000139975863</v>
+        <v>-1635.000153623408</v>
       </c>
       <c r="C11">
-        <v>-1635.000139975863</v>
+        <v>-1635.000153623408</v>
       </c>
       <c r="D11">
         <v>0</v>
       </c>
       <c r="E11">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="F11" t="s">
         <v>6</v>
@@ -2353,16 +2353,16 @@
         <v>10</v>
       </c>
       <c r="B12">
-        <v>-2002.000101219678</v>
+        <v>-2002.000093729689</v>
       </c>
       <c r="C12">
-        <v>-2002.000101219678</v>
+        <v>-2002.000093729689</v>
       </c>
       <c r="D12">
         <v>0</v>
       </c>
       <c r="E12">
-        <v>272</v>
+        <v>86</v>
       </c>
       <c r="F12" t="s">
         <v>6</v>
@@ -2373,13 +2373,13 @@
         <v>9</v>
       </c>
       <c r="B13">
-        <v>-2218.000119539372</v>
+        <v>-2218.000126301951</v>
       </c>
       <c r="C13">
-        <v>-2244.999999999996</v>
+        <v>-2283.660573023993</v>
       </c>
       <c r="D13">
-        <v>1.202667281096855</v>
+        <v>2.87522793438149</v>
       </c>
       <c r="E13">
         <v>300</v>
@@ -2393,13 +2393,13 @@
         <v>8</v>
       </c>
       <c r="B14">
-        <v>-2587.000126164291</v>
+        <v>-2587.000132690505</v>
       </c>
       <c r="C14">
-        <v>-2668.427914110429</v>
+        <v>-2668.522616218312</v>
       </c>
       <c r="D14">
-        <v>3.051526612937709</v>
+        <v>3.05496693310157</v>
       </c>
       <c r="E14">
         <v>300</v>
@@ -2413,13 +2413,13 @@
         <v>7</v>
       </c>
       <c r="B15">
-        <v>-2937.500191458481</v>
+        <v>-2937.500197775225</v>
       </c>
       <c r="C15">
-        <v>-3623.999577992986</v>
+        <v>-4819.571873825887</v>
       </c>
       <c r="D15">
-        <v>18.9431420109242</v>
+        <v>39.05059879429976</v>
       </c>
       <c r="E15">
         <v>300</v>
@@ -2433,13 +2433,13 @@
         <v>6</v>
       </c>
       <c r="B16">
-        <v>-3499.000214551427</v>
+        <v>-3499.000244503402</v>
       </c>
       <c r="C16">
-        <v>-8716.897339435807</v>
+        <v>-8717.969452569449</v>
       </c>
       <c r="D16">
-        <v>59.85956839572123</v>
+        <v>59.86450441768706</v>
       </c>
       <c r="E16">
         <v>300</v>
@@ -2453,13 +2453,13 @@
         <v>5</v>
       </c>
       <c r="B17">
-        <v>-4210.000164221095</v>
+        <v>-4211.000233963527</v>
       </c>
       <c r="C17">
-        <v>-10821.67346924542</v>
+        <v>-10786.67346906201</v>
       </c>
       <c r="D17">
-        <v>61.09658846955903</v>
+        <v>60.96108549089409</v>
       </c>
       <c r="E17">
         <v>300</v>
@@ -2473,13 +2473,13 @@
         <v>4</v>
       </c>
       <c r="B18">
-        <v>-4942.000224494345</v>
+        <v>-4763.000303802989</v>
       </c>
       <c r="C18">
-        <v>-13791.7959151268</v>
+        <v>-14002.51019287109</v>
       </c>
       <c r="D18">
-        <v>64.16710155148124</v>
+        <v>65.98466819022269</v>
       </c>
       <c r="E18">
         <v>300</v>
@@ -2493,16 +2493,16 @@
         <v>3</v>
       </c>
       <c r="B19">
-        <v>-6164.000406323416</v>
+        <v>-6371.000560503014</v>
       </c>
       <c r="C19">
-        <v>-19013.22448972139</v>
+        <v>-19213.9387754456</v>
       </c>
       <c r="D19">
-        <v>67.58045743553023</v>
+        <v>66.84177755034374</v>
       </c>
       <c r="E19">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="F19" t="s">
         <v>7</v>
@@ -2513,13 +2513,13 @@
         <v>2</v>
       </c>
       <c r="B20">
-        <v>-7701.000708818346</v>
+        <v>-7850.000580349149</v>
       </c>
       <c r="C20">
-        <v>-23307.22222222221</v>
+        <v>-23312.22222222222</v>
       </c>
       <c r="D20">
-        <v>66.95873650067212</v>
+        <v>66.32667402738556</v>
       </c>
       <c r="E20">
         <v>300</v>
@@ -2533,13 +2533,13 @@
         <v>1</v>
       </c>
       <c r="B21">
-        <v>-13019.00142282512</v>
+        <v>-13019.00133960905</v>
       </c>
       <c r="C21">
-        <v>-22577.22222221948</v>
+        <v>-22577.22222222222</v>
       </c>
       <c r="D21">
-        <v>42.33568109183773</v>
+        <v>42.3356814604289</v>
       </c>
       <c r="E21">
         <v>300</v>

</xml_diff>

<commit_message>
Updated results with 300 and 3600 s time limits
</commit_message>
<xml_diff>
--- a/hexaly_benchmarking_results/known_n.xlsx
+++ b/hexaly_benchmarking_results/known_n.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="10">
   <si>
     <t>Accuracy</t>
   </si>
@@ -473,13 +473,13 @@
         <v>40</v>
       </c>
       <c r="B4">
-        <v>-145.0000000000001</v>
+        <v>-144.9962316132948</v>
       </c>
       <c r="C4">
-        <v>-145.0000000000001</v>
+        <v>-145.0006453098344</v>
       </c>
       <c r="D4">
-        <v>0</v>
+        <v>0.003043915101371185</v>
       </c>
       <c r="E4">
         <v>0</v>
@@ -496,10 +496,10 @@
         <v>-451</v>
       </c>
       <c r="C5">
-        <v>-451</v>
+        <v>-451.0000000000001</v>
       </c>
       <c r="D5">
-        <v>0</v>
+        <v>2.520772455024745E-14</v>
       </c>
       <c r="E5">
         <v>0</v>
@@ -536,10 +536,10 @@
         <v>-868</v>
       </c>
       <c r="C7">
-        <v>-868.0202623340165</v>
+        <v>-868</v>
       </c>
       <c r="D7">
-        <v>0.002334315786822284</v>
+        <v>0</v>
       </c>
       <c r="E7">
         <v>0</v>
@@ -553,13 +553,13 @@
         <v>17</v>
       </c>
       <c r="B8">
-        <v>-1060.500000000016</v>
+        <v>-1060.5</v>
       </c>
       <c r="C8">
-        <v>-1060.500000000355</v>
+        <v>-1060.5</v>
       </c>
       <c r="D8">
-        <v>3.194594779917985E-11</v>
+        <v>0</v>
       </c>
       <c r="E8">
         <v>0</v>
@@ -573,10 +573,10 @@
         <v>15</v>
       </c>
       <c r="B9">
-        <v>-1254.000000000001</v>
+        <v>-1254</v>
       </c>
       <c r="C9">
-        <v>-1254.000000000001</v>
+        <v>-1254</v>
       </c>
       <c r="D9">
         <v>0</v>
@@ -613,13 +613,13 @@
         <v>12</v>
       </c>
       <c r="B11">
-        <v>-1634.999999999998</v>
+        <v>-1635</v>
       </c>
       <c r="C11">
-        <v>-1635.000000000048</v>
+        <v>-1635.000001771195</v>
       </c>
       <c r="D11">
-        <v>3.101182239990168E-12</v>
+        <v>1.083299694374069E-07</v>
       </c>
       <c r="E11">
         <v>0</v>
@@ -653,10 +653,10 @@
         <v>9</v>
       </c>
       <c r="B13">
-        <v>-2218.000000000007</v>
+        <v>-2218</v>
       </c>
       <c r="C13">
-        <v>-2218.000000000007</v>
+        <v>-2218</v>
       </c>
       <c r="D13">
         <v>0</v>
@@ -673,10 +673,10 @@
         <v>8</v>
       </c>
       <c r="B14">
-        <v>-2587</v>
+        <v>-2587.000000000352</v>
       </c>
       <c r="C14">
-        <v>-2587</v>
+        <v>-2587.000000000352</v>
       </c>
       <c r="D14">
         <v>0</v>
@@ -693,13 +693,13 @@
         <v>7</v>
       </c>
       <c r="B15">
-        <v>-2937.500157055813</v>
+        <v>-2894.000061125766</v>
       </c>
       <c r="C15">
-        <v>-11664.00000000002</v>
+        <v>-11694.00000000002</v>
       </c>
       <c r="D15">
-        <v>74.81567080713471</v>
+        <v>75.252265596667</v>
       </c>
       <c r="E15">
         <v>300</v>
@@ -713,13 +713,13 @@
         <v>6</v>
       </c>
       <c r="B16">
-        <v>-3499.000255781522</v>
+        <v>-3318.000175119152</v>
       </c>
       <c r="C16">
-        <v>-14187.00000000003</v>
+        <v>-14177.00000000003</v>
       </c>
       <c r="D16">
-        <v>75.33657393542316</v>
+        <v>76.59589352388274</v>
       </c>
       <c r="E16">
         <v>300</v>
@@ -733,13 +733,13 @@
         <v>5</v>
       </c>
       <c r="B17">
-        <v>-4211.000243740127</v>
+        <v>-4231.000260503773</v>
       </c>
       <c r="C17">
-        <v>-17531.00000000004</v>
+        <v>-17571.00000000004</v>
       </c>
       <c r="D17">
-        <v>75.97969172471555</v>
+        <v>75.92054942516782</v>
       </c>
       <c r="E17">
         <v>300</v>
@@ -753,13 +753,13 @@
         <v>4</v>
       </c>
       <c r="B18">
-        <v>-4763.000289078626</v>
+        <v>-4488.000870768987</v>
       </c>
       <c r="C18">
-        <v>-19539.00000000002</v>
+        <v>-19504.00000000002</v>
       </c>
       <c r="D18">
-        <v>75.62311126936578</v>
+        <v>76.98933105635264</v>
       </c>
       <c r="E18">
         <v>300</v>
@@ -773,13 +773,13 @@
         <v>3</v>
       </c>
       <c r="B19">
-        <v>-6371.000435102151</v>
+        <v>-6210.997926318658</v>
       </c>
       <c r="C19">
-        <v>-20739.00000000004</v>
+        <v>-20644.00000000004</v>
       </c>
       <c r="D19">
-        <v>69.28009819614186</v>
+        <v>69.91378644488158</v>
       </c>
       <c r="E19">
         <v>300</v>
@@ -793,13 +793,13 @@
         <v>2</v>
       </c>
       <c r="B20">
-        <v>-7818.000162787889</v>
+        <v>-7697.000682962473</v>
       </c>
       <c r="C20">
-        <v>-23598.00000000009</v>
+        <v>-23613.00000000009</v>
       </c>
       <c r="D20">
-        <v>66.87007304522477</v>
+        <v>67.40354600024374</v>
       </c>
       <c r="E20">
         <v>300</v>
@@ -813,13 +813,13 @@
         <v>1</v>
       </c>
       <c r="B21">
-        <v>-11068.10121677245</v>
+        <v>-9746.286110952917</v>
       </c>
       <c r="C21">
-        <v>-25755</v>
+        <v>-25760</v>
       </c>
       <c r="D21">
-        <v>57.02542723054766</v>
+        <v>62.16503838915794</v>
       </c>
       <c r="E21">
         <v>300</v>
@@ -886,10 +886,10 @@
         <v>-86</v>
       </c>
       <c r="C3">
-        <v>-86.00000000000001</v>
+        <v>-86.00000000000006</v>
       </c>
       <c r="D3">
-        <v>1.652424966883954E-14</v>
+        <v>6.609699867535812E-14</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -903,13 +903,13 @@
         <v>40</v>
       </c>
       <c r="B4">
-        <v>-145.0000035456657</v>
+        <v>-145</v>
       </c>
       <c r="C4">
-        <v>-145.0000035456657</v>
+        <v>-145.0000038867176</v>
       </c>
       <c r="D4">
-        <v>0</v>
+        <v>2.680494800344536E-06</v>
       </c>
       <c r="E4">
         <v>0</v>
@@ -923,13 +923,13 @@
         <v>30</v>
       </c>
       <c r="B5">
-        <v>-451</v>
+        <v>-450.9999999999995</v>
       </c>
       <c r="C5">
-        <v>-451.0000000000001</v>
+        <v>-451.0000070095472</v>
       </c>
       <c r="D5">
-        <v>1.260386227512373E-14</v>
+        <v>1.554223409807457E-06</v>
       </c>
       <c r="E5">
         <v>0</v>
@@ -943,13 +943,13 @@
         <v>24</v>
       </c>
       <c r="B6">
-        <v>-658.9999999999989</v>
+        <v>-658.9997682152291</v>
       </c>
       <c r="C6">
-        <v>-659.0000000004791</v>
+        <v>-659.0000000000084</v>
       </c>
       <c r="D6">
-        <v>7.28699852102818E-11</v>
+        <v>3.517219716487252E-05</v>
       </c>
       <c r="E6">
         <v>0</v>
@@ -963,13 +963,13 @@
         <v>20</v>
       </c>
       <c r="B7">
-        <v>-868.0000000043406</v>
+        <v>-868.0000110654701</v>
       </c>
       <c r="C7">
-        <v>-868.0000083491861</v>
+        <v>-868.0000129164089</v>
       </c>
       <c r="D7">
-        <v>9.613877306767098E-07</v>
+        <v>2.132417958534078E-07</v>
       </c>
       <c r="E7">
         <v>1</v>
@@ -983,13 +983,13 @@
         <v>17</v>
       </c>
       <c r="B8">
-        <v>-1060.500012055399</v>
+        <v>-1060.500016980288</v>
       </c>
       <c r="C8">
-        <v>-1060.500016475598</v>
+        <v>-1060.500019456169</v>
       </c>
       <c r="D8">
-        <v>4.168032769097318E-07</v>
+        <v>2.334635979417868E-07</v>
       </c>
       <c r="E8">
         <v>4</v>
@@ -1003,16 +1003,16 @@
         <v>15</v>
       </c>
       <c r="B9">
-        <v>-1254.000006284345</v>
+        <v>-1254.000010916349</v>
       </c>
       <c r="C9">
-        <v>-1254.000010053599</v>
+        <v>-1254.000010916349</v>
       </c>
       <c r="D9">
-        <v>3.005784772933242E-07</v>
+        <v>0</v>
       </c>
       <c r="E9">
-        <v>20</v>
+        <v>39</v>
       </c>
       <c r="F9" t="s">
         <v>6</v>
@@ -1023,16 +1023,16 @@
         <v>13</v>
       </c>
       <c r="B10">
-        <v>-1449.000010879016</v>
+        <v>-1449.000010282142</v>
       </c>
       <c r="C10">
-        <v>-1449.000010879016</v>
+        <v>-1449.000010282142</v>
       </c>
       <c r="D10">
         <v>0</v>
       </c>
       <c r="E10">
-        <v>64</v>
+        <v>45</v>
       </c>
       <c r="F10" t="s">
         <v>6</v>
@@ -1043,19 +1043,19 @@
         <v>12</v>
       </c>
       <c r="B11">
-        <v>-1635.00002838934</v>
+        <v>-1635.000028851072</v>
       </c>
       <c r="C11">
-        <v>-1635.00002838934</v>
+        <v>-1642.999999999844</v>
       </c>
       <c r="D11">
-        <v>0</v>
+        <v>0.4869124253665659</v>
       </c>
       <c r="E11">
-        <v>263</v>
+        <v>300</v>
       </c>
       <c r="F11" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -1063,13 +1063,13 @@
         <v>10</v>
       </c>
       <c r="B12">
-        <v>-2002.000007198596</v>
+        <v>-2001.999817202687</v>
       </c>
       <c r="C12">
-        <v>-2469.999999999876</v>
+        <v>-2469.999999999987</v>
       </c>
       <c r="D12">
-        <v>18.94736812960744</v>
+        <v>18.94737582175313</v>
       </c>
       <c r="E12">
         <v>300</v>
@@ -1083,13 +1083,13 @@
         <v>9</v>
       </c>
       <c r="B13">
-        <v>-2214.792097351755</v>
+        <v>-2156.459415704963</v>
       </c>
       <c r="C13">
-        <v>-2517.999999999934</v>
+        <v>-2517.999999999048</v>
       </c>
       <c r="D13">
-        <v>12.04161646736246</v>
+        <v>14.35824401486186</v>
       </c>
       <c r="E13">
         <v>300</v>
@@ -1103,13 +1103,13 @@
         <v>8</v>
       </c>
       <c r="B14">
-        <v>-2587.000007165996</v>
+        <v>-2587.000007199757</v>
       </c>
       <c r="C14">
-        <v>-3234.999999998702</v>
+        <v>-3234.999999968822</v>
       </c>
       <c r="D14">
-        <v>20.03091167953527</v>
+        <v>20.030911677753</v>
       </c>
       <c r="E14">
         <v>300</v>
@@ -1123,13 +1123,13 @@
         <v>7</v>
       </c>
       <c r="B15">
-        <v>-2934.262868179775</v>
+        <v>-2965.114339026486</v>
       </c>
       <c r="C15">
-        <v>-3371.999999999989</v>
+        <v>-3329.999999999942</v>
       </c>
       <c r="D15">
-        <v>12.98152822717129</v>
+        <v>10.95752735656044</v>
       </c>
       <c r="E15">
         <v>300</v>
@@ -1143,13 +1143,13 @@
         <v>6</v>
       </c>
       <c r="B16">
-        <v>-3499.000010613431</v>
+        <v>-3453.000011170847</v>
       </c>
       <c r="C16">
-        <v>-7593.576308782231</v>
+        <v>-13661.68341904866</v>
       </c>
       <c r="D16">
-        <v>53.92157965718053</v>
+        <v>74.72493026477042</v>
       </c>
       <c r="E16">
         <v>300</v>
@@ -1163,13 +1163,13 @@
         <v>5</v>
       </c>
       <c r="B17">
-        <v>-4211.000007167921</v>
+        <v>-4231.000010940826</v>
       </c>
       <c r="C17">
-        <v>-27075</v>
+        <v>-27115</v>
       </c>
       <c r="D17">
-        <v>84.44690671406123</v>
+        <v>84.39609068434142</v>
       </c>
       <c r="E17">
         <v>300</v>
@@ -1183,13 +1183,13 @@
         <v>4</v>
       </c>
       <c r="B18">
-        <v>-4763.000007070595</v>
+        <v>-4581.757671894174</v>
       </c>
       <c r="C18">
-        <v>-27015</v>
+        <v>-26980</v>
       </c>
       <c r="D18">
-        <v>82.36905420295912</v>
+        <v>83.01794784323879</v>
       </c>
       <c r="E18">
         <v>300</v>
@@ -1203,13 +1203,13 @@
         <v>3</v>
       </c>
       <c r="B19">
-        <v>-6344.000002643128</v>
+        <v>-6740.000003962358</v>
       </c>
       <c r="C19">
-        <v>-26655</v>
+        <v>-26560</v>
       </c>
       <c r="D19">
-        <v>76.19958730953618</v>
+        <v>74.6234939609851</v>
       </c>
       <c r="E19">
         <v>300</v>
@@ -1223,19 +1223,19 @@
         <v>2</v>
       </c>
       <c r="B20">
-        <v>-7567.83261715334</v>
+        <v>41.00000000016053</v>
       </c>
       <c r="C20">
-        <v>-26490</v>
-      </c>
-      <c r="D20">
-        <v>71.43136044864727</v>
+        <v>-26505</v>
+      </c>
+      <c r="D20" t="s">
+        <v>8</v>
       </c>
       <c r="E20">
         <v>300</v>
       </c>
       <c r="F20" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="21" spans="1:6">
@@ -1243,10 +1243,10 @@
         <v>1</v>
       </c>
       <c r="B21">
-        <v>877</v>
+        <v>908</v>
       </c>
       <c r="C21">
-        <v>-25755</v>
+        <v>-25760</v>
       </c>
       <c r="D21" t="s">
         <v>8</v>
@@ -1336,10 +1336,10 @@
         <v>-145.0000000000001</v>
       </c>
       <c r="C4">
-        <v>-145.0000000000001</v>
+        <v>-145.0000024860404</v>
       </c>
       <c r="D4">
-        <v>0</v>
+        <v>1.714510543046501E-06</v>
       </c>
       <c r="E4">
         <v>0</v>
@@ -1373,13 +1373,13 @@
         <v>24</v>
       </c>
       <c r="B6">
-        <v>-659.0000000000005</v>
+        <v>-659.0000000000176</v>
       </c>
       <c r="C6">
-        <v>-659.0000000000006</v>
+        <v>-659.0000000000176</v>
       </c>
       <c r="D6">
-        <v>1.725141695320424E-14</v>
+        <v>0</v>
       </c>
       <c r="E6">
         <v>0</v>
@@ -1393,16 +1393,16 @@
         <v>20</v>
       </c>
       <c r="B7">
-        <v>-868.0000160197219</v>
+        <v>-868.0000194616252</v>
       </c>
       <c r="C7">
-        <v>-868.0000160197219</v>
+        <v>-868.0000194616252</v>
       </c>
       <c r="D7">
         <v>0</v>
       </c>
       <c r="E7">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="F7" t="s">
         <v>6</v>
@@ -1413,16 +1413,16 @@
         <v>17</v>
       </c>
       <c r="B8">
-        <v>-1060.500018879588</v>
+        <v>-1060.500019815555</v>
       </c>
       <c r="C8">
-        <v>-1060.500018879588</v>
+        <v>-1060.500019815555</v>
       </c>
       <c r="D8">
         <v>0</v>
       </c>
       <c r="E8">
-        <v>175</v>
+        <v>230</v>
       </c>
       <c r="F8" t="s">
         <v>6</v>
@@ -1433,13 +1433,13 @@
         <v>15</v>
       </c>
       <c r="B9">
-        <v>-1254.000011184923</v>
+        <v>-1254.000007393707</v>
       </c>
       <c r="C9">
-        <v>-1262</v>
+        <v>-1262.841149944514</v>
       </c>
       <c r="D9">
-        <v>0.6339135352676194</v>
+        <v>0.7000993395879812</v>
       </c>
       <c r="E9">
         <v>300</v>
@@ -1453,13 +1453,13 @@
         <v>13</v>
       </c>
       <c r="B10">
-        <v>-1449.000011171598</v>
+        <v>-1449.0000111403</v>
       </c>
       <c r="C10">
-        <v>-1704.999999999796</v>
+        <v>-1452.9999999997</v>
       </c>
       <c r="D10">
-        <v>15.01466210136237</v>
+        <v>0.2752917315485453</v>
       </c>
       <c r="E10">
         <v>300</v>
@@ -1473,13 +1473,13 @@
         <v>12</v>
       </c>
       <c r="B11">
-        <v>-1635.000028908659</v>
+        <v>-1635.000028257185</v>
       </c>
       <c r="C11">
-        <v>-1700</v>
+        <v>-1728.864489060958</v>
       </c>
       <c r="D11">
-        <v>3.823527711255377</v>
+        <v>5.429254947260557</v>
       </c>
       <c r="E11">
         <v>300</v>
@@ -1493,13 +1493,13 @@
         <v>10</v>
       </c>
       <c r="B12">
-        <v>-2001.999848598414</v>
+        <v>-2001.999945525726</v>
       </c>
       <c r="C12">
-        <v>-2937.802959907597</v>
+        <v>-3800.525682538792</v>
       </c>
       <c r="D12">
-        <v>31.85384193835167</v>
+        <v>47.32307810143862</v>
       </c>
       <c r="E12">
         <v>300</v>
@@ -1513,13 +1513,13 @@
         <v>9</v>
       </c>
       <c r="B13">
-        <v>-2218.000011088411</v>
+        <v>-2217.999441172387</v>
       </c>
       <c r="C13">
-        <v>-4036.718166019533</v>
+        <v>-4142.581582910376</v>
       </c>
       <c r="D13">
-        <v>45.05437536464172</v>
+        <v>46.45852117137717</v>
       </c>
       <c r="E13">
         <v>300</v>
@@ -1533,13 +1533,13 @@
         <v>8</v>
       </c>
       <c r="B14">
-        <v>-2587.000007184351</v>
+        <v>-2587.000007136976</v>
       </c>
       <c r="C14">
-        <v>-7763.619539464617</v>
+        <v>-8032.006428749053</v>
       </c>
       <c r="D14">
-        <v>66.67791364538257</v>
+        <v>67.79136035203736</v>
       </c>
       <c r="E14">
         <v>300</v>
@@ -1553,13 +1553,13 @@
         <v>7</v>
       </c>
       <c r="B15">
-        <v>-2933.406112432342</v>
+        <v>-2962.537773633487</v>
       </c>
       <c r="C15">
-        <v>-10041.83681899469</v>
+        <v>-10104.61835515283</v>
       </c>
       <c r="D15">
-        <v>70.78815195559001</v>
+        <v>70.68134916621817</v>
       </c>
       <c r="E15">
         <v>300</v>
@@ -1573,13 +1573,13 @@
         <v>6</v>
       </c>
       <c r="B16">
-        <v>-3499.000011151707</v>
+        <v>-3453.000010129845</v>
       </c>
       <c r="C16">
-        <v>-17097.52069760642</v>
+        <v>-15585.02908643527</v>
       </c>
       <c r="D16">
-        <v>79.53504444862844</v>
+        <v>77.84412213169861</v>
       </c>
       <c r="E16">
         <v>300</v>
@@ -1593,13 +1593,13 @@
         <v>5</v>
       </c>
       <c r="B17">
-        <v>-4211.000007079504</v>
+        <v>-4231.0000100803</v>
       </c>
       <c r="C17">
-        <v>-23291.02659388755</v>
+        <v>-22518.97368603328</v>
       </c>
       <c r="D17">
-        <v>81.92007557028582</v>
+        <v>81.2113994666442</v>
       </c>
       <c r="E17">
         <v>300</v>
@@ -1613,13 +1613,13 @@
         <v>4</v>
       </c>
       <c r="B18">
-        <v>-4763.000006256601</v>
+        <v>-4808.490551152878</v>
       </c>
       <c r="C18">
-        <v>-27015</v>
+        <v>-26980</v>
       </c>
       <c r="D18">
-        <v>82.36905420597222</v>
+        <v>82.17757393938889</v>
       </c>
       <c r="E18">
         <v>300</v>
@@ -1633,13 +1633,13 @@
         <v>3</v>
       </c>
       <c r="B19">
-        <v>-6371.000010875239</v>
+        <v>-6740.000003997709</v>
       </c>
       <c r="C19">
-        <v>-26655</v>
+        <v>-26560</v>
       </c>
       <c r="D19">
-        <v>76.0982929623889</v>
+        <v>74.62349396085199</v>
       </c>
       <c r="E19">
         <v>300</v>
@@ -1653,13 +1653,13 @@
         <v>2</v>
       </c>
       <c r="B20">
-        <v>-7850.000005262159</v>
+        <v>-7697.000004047792</v>
       </c>
       <c r="C20">
-        <v>-26490</v>
+        <v>-26505</v>
       </c>
       <c r="D20">
-        <v>70.36617589557508</v>
+        <v>70.96019617412644</v>
       </c>
       <c r="E20">
         <v>300</v>
@@ -1673,13 +1673,13 @@
         <v>1</v>
       </c>
       <c r="B21">
-        <v>-13018.99984637278</v>
+        <v>-12736.00000645221</v>
       </c>
       <c r="C21">
-        <v>-25755</v>
+        <v>-25760</v>
       </c>
       <c r="D21">
-        <v>49.45059271453008</v>
+        <v>50.55900618613273</v>
       </c>
       <c r="E21">
         <v>300</v>
@@ -1743,13 +1743,13 @@
         <v>60</v>
       </c>
       <c r="B3">
-        <v>-86.00000000000003</v>
+        <v>-86</v>
       </c>
       <c r="C3">
-        <v>-86.00000000000003</v>
+        <v>-86.00000000000001</v>
       </c>
       <c r="D3">
-        <v>0</v>
+        <v>1.652424966883954E-14</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -1766,10 +1766,10 @@
         <v>-145.0000000000001</v>
       </c>
       <c r="C4">
-        <v>-145.0004439845235</v>
+        <v>-145.0004439845237</v>
       </c>
       <c r="D4">
-        <v>0.0003061952855351152</v>
+        <v>0.0003061952856135194</v>
       </c>
       <c r="E4">
         <v>0</v>
@@ -1783,13 +1783,13 @@
         <v>30</v>
       </c>
       <c r="B5">
-        <v>-450.9995000645418</v>
+        <v>-450.9861740828734</v>
       </c>
       <c r="C5">
-        <v>-451.0001483518363</v>
+        <v>-451.0001483518368</v>
       </c>
       <c r="D5">
-        <v>0.0001437443639257585</v>
+        <v>0.003098506511454737</v>
       </c>
       <c r="E5">
         <v>0</v>
@@ -1823,13 +1823,13 @@
         <v>20</v>
       </c>
       <c r="B7">
-        <v>-868</v>
+        <v>-867.9999999999998</v>
       </c>
       <c r="C7">
-        <v>-868</v>
+        <v>-867.9999999999999</v>
       </c>
       <c r="D7">
-        <v>0</v>
+        <v>1.309756194949494E-14</v>
       </c>
       <c r="E7">
         <v>0</v>
@@ -1843,16 +1843,16 @@
         <v>17</v>
       </c>
       <c r="B8">
-        <v>-1060.499999999991</v>
+        <v>-1060.5</v>
       </c>
       <c r="C8">
-        <v>-1060.499999999991</v>
+        <v>-1060.5</v>
       </c>
       <c r="D8">
         <v>0</v>
       </c>
       <c r="E8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F8" t="s">
         <v>6</v>
@@ -1863,10 +1863,10 @@
         <v>15</v>
       </c>
       <c r="B9">
-        <v>-1253.999999999999</v>
+        <v>-1254</v>
       </c>
       <c r="C9">
-        <v>-1253.999999999999</v>
+        <v>-1254</v>
       </c>
       <c r="D9">
         <v>0</v>
@@ -1892,7 +1892,7 @@
         <v>0</v>
       </c>
       <c r="E10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F10" t="s">
         <v>6</v>
@@ -1903,16 +1903,16 @@
         <v>12</v>
       </c>
       <c r="B11">
-        <v>-1635.000000000205</v>
+        <v>-1635</v>
       </c>
       <c r="C11">
-        <v>-1635.000000000205</v>
+        <v>-1635</v>
       </c>
       <c r="D11">
         <v>0</v>
       </c>
       <c r="E11">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F11" t="s">
         <v>6</v>
@@ -1932,7 +1932,7 @@
         <v>0</v>
       </c>
       <c r="E12">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F12" t="s">
         <v>6</v>
@@ -1952,7 +1952,7 @@
         <v>0</v>
       </c>
       <c r="E13">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="F13" t="s">
         <v>6</v>
@@ -1972,7 +1972,7 @@
         <v>0</v>
       </c>
       <c r="E14">
-        <v>34</v>
+        <v>25</v>
       </c>
       <c r="F14" t="s">
         <v>6</v>
@@ -1983,16 +1983,16 @@
         <v>7</v>
       </c>
       <c r="B15">
-        <v>-2937.5</v>
+        <v>-2966.000156468799</v>
       </c>
       <c r="C15">
-        <v>-2937.5</v>
+        <v>-2966.00015959707</v>
       </c>
       <c r="D15">
-        <v>0</v>
+        <v>1.054710530189852E-07</v>
       </c>
       <c r="E15">
-        <v>94</v>
+        <v>19</v>
       </c>
       <c r="F15" t="s">
         <v>6</v>
@@ -2003,16 +2003,16 @@
         <v>6</v>
       </c>
       <c r="B16">
-        <v>-3499.000241669576</v>
+        <v>-3453</v>
       </c>
       <c r="C16">
-        <v>-3499.000244261619</v>
+        <v>-3453</v>
       </c>
       <c r="D16">
-        <v>7.407952096901042E-08</v>
+        <v>0</v>
       </c>
       <c r="E16">
-        <v>25</v>
+        <v>154</v>
       </c>
       <c r="F16" t="s">
         <v>6</v>
@@ -2023,19 +2023,19 @@
         <v>5</v>
       </c>
       <c r="B17">
-        <v>-4119.000348170899</v>
+        <v>-4231.00033152282</v>
       </c>
       <c r="C17">
-        <v>-4210.99999999377</v>
+        <v>-4231.00033152282</v>
       </c>
       <c r="D17">
-        <v>2.184745946877392</v>
+        <v>0</v>
       </c>
       <c r="E17">
-        <v>300</v>
+        <v>66</v>
       </c>
       <c r="F17" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="18" spans="1:6">
@@ -2043,19 +2043,19 @@
         <v>4</v>
       </c>
       <c r="B18">
-        <v>-4763.000320036102</v>
+        <v>-4594.125385118025</v>
       </c>
       <c r="C18">
-        <v>-4763.000320036102</v>
+        <v>-4831.04294478526</v>
       </c>
       <c r="D18">
-        <v>0</v>
+        <v>4.904066520935591</v>
       </c>
       <c r="E18">
-        <v>246</v>
+        <v>300</v>
       </c>
       <c r="F18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="19" spans="1:6">
@@ -2063,13 +2063,13 @@
         <v>3</v>
       </c>
       <c r="B19">
-        <v>-6191.000473068396</v>
+        <v>-6632.000422204775</v>
       </c>
       <c r="C19">
-        <v>-19213.93877550212</v>
+        <v>-6739.999999996653</v>
       </c>
       <c r="D19">
-        <v>67.77859789497218</v>
+        <v>1.602367623025698</v>
       </c>
       <c r="E19">
         <v>300</v>
@@ -2083,19 +2083,19 @@
         <v>2</v>
       </c>
       <c r="B20">
-        <v>-4114.087816757833</v>
+        <v>-2894.450822338931</v>
       </c>
       <c r="C20">
-        <v>-23598.00000000009</v>
-      </c>
-      <c r="D20">
-        <v>82.5659470431485</v>
+        <v>-23613.00000000009</v>
+      </c>
+      <c r="D20" t="s">
+        <v>8</v>
       </c>
       <c r="E20">
         <v>300</v>
       </c>
       <c r="F20" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="21" spans="1:6">
@@ -2103,10 +2103,10 @@
         <v>1</v>
       </c>
       <c r="B21">
-        <v>2245</v>
+        <v>2240</v>
       </c>
       <c r="C21">
-        <v>-25755</v>
+        <v>-25760</v>
       </c>
       <c r="D21" t="s">
         <v>8</v>
@@ -2196,10 +2196,10 @@
         <v>-145.0000000000001</v>
       </c>
       <c r="C4">
-        <v>-145.0000008254828</v>
+        <v>-145.0000000000001</v>
       </c>
       <c r="D4">
-        <v>5.692984601490828E-07</v>
+        <v>3.920235783503998E-14</v>
       </c>
       <c r="E4">
         <v>0</v>
@@ -2236,10 +2236,10 @@
         <v>-659</v>
       </c>
       <c r="C6">
-        <v>-659</v>
+        <v>-659.0000000000107</v>
       </c>
       <c r="D6">
-        <v>0</v>
+        <v>1.621633193601173E-12</v>
       </c>
       <c r="E6">
         <v>0</v>
@@ -2253,13 +2253,13 @@
         <v>20</v>
       </c>
       <c r="B7">
-        <v>-868.000000000001</v>
+        <v>-868.0000000000003</v>
       </c>
       <c r="C7">
-        <v>-868.0000105198319</v>
+        <v>-868.0000136837932</v>
       </c>
       <c r="D7">
-        <v>1.211962068282054E-06</v>
+        <v>1.576473808343545E-06</v>
       </c>
       <c r="E7">
         <v>1</v>
@@ -2273,16 +2273,16 @@
         <v>17</v>
       </c>
       <c r="B8">
-        <v>-1060.500038374746</v>
+        <v>-1060.50004974893</v>
       </c>
       <c r="C8">
-        <v>-1060.500038374746</v>
+        <v>-1060.50004974893</v>
       </c>
       <c r="D8">
         <v>0</v>
       </c>
       <c r="E8">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="F8" t="s">
         <v>6</v>
@@ -2293,16 +2293,16 @@
         <v>15</v>
       </c>
       <c r="B9">
-        <v>-1254</v>
+        <v>-1254.000050429609</v>
       </c>
       <c r="C9">
-        <v>-1254</v>
+        <v>-1254.000050429609</v>
       </c>
       <c r="D9">
         <v>0</v>
       </c>
       <c r="E9">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="F9" t="s">
         <v>6</v>
@@ -2313,16 +2313,16 @@
         <v>13</v>
       </c>
       <c r="B10">
-        <v>-1449.000083030363</v>
+        <v>-1449.000071044483</v>
       </c>
       <c r="C10">
-        <v>-1449.000083030363</v>
+        <v>-1449.000071044483</v>
       </c>
       <c r="D10">
         <v>0</v>
       </c>
       <c r="E10">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="F10" t="s">
         <v>6</v>
@@ -2333,16 +2333,16 @@
         <v>12</v>
       </c>
       <c r="B11">
-        <v>-1635.000153623408</v>
+        <v>-1635.000156468598</v>
       </c>
       <c r="C11">
-        <v>-1635.000153623408</v>
+        <v>-1635.000156468598</v>
       </c>
       <c r="D11">
         <v>0</v>
       </c>
       <c r="E11">
-        <v>91</v>
+        <v>82</v>
       </c>
       <c r="F11" t="s">
         <v>6</v>
@@ -2353,16 +2353,16 @@
         <v>10</v>
       </c>
       <c r="B12">
-        <v>-2002.000093729689</v>
+        <v>-2002.000095562462</v>
       </c>
       <c r="C12">
-        <v>-2002.000093729689</v>
+        <v>-2002.000095562462</v>
       </c>
       <c r="D12">
         <v>0</v>
       </c>
       <c r="E12">
-        <v>86</v>
+        <v>127</v>
       </c>
       <c r="F12" t="s">
         <v>6</v>
@@ -2373,13 +2373,13 @@
         <v>9</v>
       </c>
       <c r="B13">
-        <v>-2218.000126301951</v>
+        <v>-2218.000122623457</v>
       </c>
       <c r="C13">
-        <v>-2283.660573023993</v>
+        <v>-2333.574039611859</v>
       </c>
       <c r="D13">
-        <v>2.87522793438149</v>
+        <v>4.952656955663818</v>
       </c>
       <c r="E13">
         <v>300</v>
@@ -2393,13 +2393,13 @@
         <v>8</v>
       </c>
       <c r="B14">
-        <v>-2587.000132690505</v>
+        <v>-2587.000140806256</v>
       </c>
       <c r="C14">
-        <v>-2668.522616218312</v>
+        <v>-2726.737522357595</v>
       </c>
       <c r="D14">
-        <v>3.05496693310157</v>
+        <v>5.124709672477696</v>
       </c>
       <c r="E14">
         <v>300</v>
@@ -2413,13 +2413,13 @@
         <v>7</v>
       </c>
       <c r="B15">
-        <v>-2937.500197775225</v>
+        <v>-2966.00018930254</v>
       </c>
       <c r="C15">
-        <v>-4819.571873825887</v>
+        <v>-3589.500000000001</v>
       </c>
       <c r="D15">
-        <v>39.05059879429976</v>
+        <v>17.37010198349244</v>
       </c>
       <c r="E15">
         <v>300</v>
@@ -2433,13 +2433,13 @@
         <v>6</v>
       </c>
       <c r="B16">
-        <v>-3499.000244503402</v>
+        <v>-3453.000214161206</v>
       </c>
       <c r="C16">
-        <v>-8717.969452569449</v>
+        <v>-8708.10076686743</v>
       </c>
       <c r="D16">
-        <v>59.86450441768706</v>
+        <v>60.34726392580141</v>
       </c>
       <c r="E16">
         <v>300</v>
@@ -2453,13 +2453,13 @@
         <v>5</v>
       </c>
       <c r="B17">
-        <v>-4211.000233963527</v>
+        <v>-4231.00026265827</v>
       </c>
       <c r="C17">
-        <v>-10786.67346906201</v>
+        <v>-10826.67346869319</v>
       </c>
       <c r="D17">
-        <v>60.96108549089409</v>
+        <v>60.92058862869757</v>
       </c>
       <c r="E17">
         <v>300</v>
@@ -2473,13 +2473,13 @@
         <v>4</v>
       </c>
       <c r="B18">
-        <v>-4763.000303802989</v>
+        <v>-4822.000350407595</v>
       </c>
       <c r="C18">
-        <v>-14002.51019287109</v>
+        <v>-13781.7959151268</v>
       </c>
       <c r="D18">
-        <v>65.98466819022269</v>
+        <v>65.01181427948008</v>
       </c>
       <c r="E18">
         <v>300</v>
@@ -2493,13 +2493,13 @@
         <v>3</v>
       </c>
       <c r="B19">
-        <v>-6371.000560503014</v>
+        <v>-6740.000246884429</v>
       </c>
       <c r="C19">
-        <v>-19213.9387754456</v>
+        <v>-18964.65306114767</v>
       </c>
       <c r="D19">
-        <v>66.84177755034374</v>
+        <v>64.46019747815757</v>
       </c>
       <c r="E19">
         <v>300</v>
@@ -2513,13 +2513,13 @@
         <v>2</v>
       </c>
       <c r="B20">
-        <v>-7850.000580349149</v>
+        <v>-7697.00060636223</v>
       </c>
       <c r="C20">
-        <v>-23312.22222222222</v>
+        <v>-23327.2222222222</v>
       </c>
       <c r="D20">
-        <v>66.32667402738556</v>
+        <v>67.00421279036884</v>
       </c>
       <c r="E20">
         <v>300</v>
@@ -2533,13 +2533,13 @@
         <v>1</v>
       </c>
       <c r="B21">
-        <v>-13019.00133960905</v>
+        <v>-12736.00152250499</v>
       </c>
       <c r="C21">
-        <v>-22577.22222222222</v>
+        <v>-22582.22222222219</v>
       </c>
       <c r="D21">
-        <v>42.3356814604289</v>
+        <v>43.60164647581919</v>
       </c>
       <c r="E21">
         <v>300</v>

</xml_diff>